<commit_message>
Fase A2: perbaikan QA ekspor (15 butir)
- ID sesi memakai tanggal lokal; konsep remedial dideduplikasi; batas
  kategori capaian tanpa celah dan teks aturan = kode.
- .xlsx: A4 lanskap, muat lebar, judul berulang; hitungan 0, capaian persen,
  tanggal Excel asli; kolom teks Uraian/Rubrik dibungkus; label (a)/(b).
- .docx: footer ID sesi + Halaman X dari Y; tabel opsi/rubrik/koreksi tidak
  terbelah; lebar kolom minimum; heading tidak melompat; skor dikoreksi
  bertanda * dengan alasan koreksi.
- Fallback .doc: page break dan paragraf gaya Word, meta charset untuk Word.
- Aturan konsistensi 6 (rujukan kriteria kasus wajib menyebut bagian);
  demo pack dan contoh skema diperbarui; CONTRACT.md dan CHANGELOG.md.
- Tes: 67 kasus PASS di selftest (suite baru Ekspor (QA A2)); contoh di
  tests/output/ dibuka ulang di Word/Excel. Keputusan D-51..D-57.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/tests/output/data-hasil-demo.xlsx
+++ b/tests/output/data-hasil-demo.xlsx
@@ -13,11 +13,23 @@
     <sheet name="Remedial" sheetId="6" r:id="rId6"/>
     <sheet name="Riwayat" sheetId="7" r:id="rId7"/>
   </sheets>
+  <definedNames>
+    <definedName name="_xlnm.Print_Titles" localSheetId="0">'Ringkasan'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="1">'PG'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="2">'Uraian'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="3">'Rubrik'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="4">'Kompetensi'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="5">'Remedial'!$1:$1</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="6">'Riwayat'!$1:$1</definedName>
+  </definedNames>
 </workbook>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <numFmts count="1">
+    <numFmt numFmtId="164" formatCode="[$-421]d mmmm yyyy hh.mm"/>
+  </numFmts>
   <fonts count="2">
     <font>
       <sz val="11"/>
@@ -72,7 +84,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top" wrapText="1"/>
@@ -89,6 +101,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="10" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -98,6 +116,9 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:C25"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -124,7 +145,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mata ujian</t>
         </is>
@@ -136,7 +157,7 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
+      <c r="A3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Versi pack</t>
         </is>
@@ -148,7 +169,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="5" t="inlineStr">
+      <c r="A4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Paket</t>
         </is>
@@ -160,7 +181,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="5" t="inlineStr">
+      <c r="A5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">ID sesi</t>
         </is>
@@ -172,7 +193,7 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="5" t="inlineStr">
+      <c r="A6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mode</t>
         </is>
@@ -184,31 +205,27 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="5" t="inlineStr">
+      <c r="A7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Mulai</t>
         </is>
       </c>
-      <c r="B7" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17 Oktober 2026 pukul 08.00</t>
-        </is>
+      <c r="B7" s="7">
+        <v>46312.33333333333</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="5" t="inlineStr">
+      <c r="A8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Dikumpulkan</t>
         </is>
       </c>
-      <c r="B8" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17 Oktober 2026 pukul 08.25</t>
-        </is>
+      <c r="B8" s="7">
+        <v>46312.350694444445</v>
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="5" t="inlineStr">
+      <c r="A9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Cara pengumpulan</t>
         </is>
@@ -220,7 +237,7 @@
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="5" t="inlineStr">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Durasi paket</t>
         </is>
@@ -232,7 +249,7 @@
       </c>
     </row>
     <row r="11">
-      <c r="A11" s="5" t="inlineStr">
+      <c r="A11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Waktu pengerjaan</t>
         </is>
@@ -244,7 +261,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="5" t="inlineStr">
+      <c r="A12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Status penilaian</t>
         </is>
@@ -256,7 +273,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+      <c r="A13" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Skor Pilihan ganda (2/2 dinilai)</t>
         </is>
@@ -269,7 +286,7 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="5" t="inlineStr">
+      <c r="A14" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Skor Numerik (1/1 dinilai)</t>
         </is>
@@ -282,7 +299,7 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="5" t="inlineStr">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Skor Esai (1/1 dinilai)</t>
         </is>
@@ -295,7 +312,7 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="5" t="inlineStr">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Skor Studi kasus (1/1 dinilai)</t>
         </is>
@@ -308,7 +325,7 @@
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
+      <c r="A17" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Skor sementara (yang sudah dinilai)</t>
         </is>
@@ -321,7 +338,7 @@
       </c>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr">
+      <c r="A18" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Nilai akhir</t>
         </is>
@@ -334,7 +351,7 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="5" t="inlineStr">
+      <c r="A19" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Passing grade</t>
         </is>
@@ -344,7 +361,7 @@
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="5" t="inlineStr">
+      <c r="A20" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Selisih terhadap passing grade</t>
         </is>
@@ -354,7 +371,7 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="5" t="inlineStr">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Status kelulusan</t>
         </is>
@@ -366,39 +383,37 @@
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="5" t="inlineStr">
+      <c r="A22" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Meninggalkan layar ujian (kali)</t>
         </is>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="23">
-      <c r="A23" s="5" t="inlineStr">
+      <c r="A23" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Koreksi manual (berlaku)</t>
         </is>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="4">
         <v>1</v>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="5" t="inlineStr">
+      <c r="A24" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Dibuat</t>
         </is>
       </c>
-      <c r="B24" s="3" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17 Oktober 2026 pukul 08.40</t>
-        </is>
+      <c r="B24" s="7">
+        <v>46312.36111111111</v>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Catatan</t>
         </is>
@@ -410,12 +425,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:S4"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -784,12 +803,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:T3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -812,7 +835,7 @@
     <col min="17" max="17" width="30" customWidth="1"/>
     <col min="18" max="18" width="12" customWidth="1"/>
     <col min="19" max="19" width="14" customWidth="1"/>
-    <col min="20" max="20" width="20" customWidth="1"/>
+    <col min="20" max="20" width="24" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -921,22 +944,22 @@
       <c r="A2" s="4">
         <v>4</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-ESA-001</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Esai</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">T02</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">K01</t>
         </is>
@@ -971,35 +994,35 @@
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membaca data dan konsep utama dengan benar.</t>
+          <t xml:space="preserve">Mengenali sifat lagging ukuran keuangan dan memberi contoh ukuran yang relevan.</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hubungan sebab-akibat dan dampak keuangan belum dijelaskan.</t>
+          <t xml:space="preserve">Hubungan sebab-akibat antarperspektif balanced scorecard belum dijelaskan.</t>
         </is>
       </c>
       <c r="O2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tunjukkan rantai sebab-akibat dan hitung dampak keputusan pada laba.</t>
-        </is>
-      </c>
-      <c r="P2" s="5" t="inlineStr">
+          <t xml:space="preserve">Gambarkan strategy map: pembelajaran -&gt; proses internal -&gt; pelanggan -&gt; keuangan.</t>
+        </is>
+      </c>
+      <c r="P2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">sedang</t>
         </is>
       </c>
-      <c r="R2" s="5" t="inlineStr">
+      <c r="R2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
       </c>
-      <c r="S2" s="5" t="inlineStr">
+      <c r="S2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
       </c>
-      <c r="T2" s="5" t="inlineStr">
+      <c r="T2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">contoh-penilai (fiktif, untuk uji)</t>
         </is>
@@ -1009,22 +1032,22 @@
       <c r="A3" s="4">
         <v>5</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-KAS-001</t>
         </is>
       </c>
-      <c r="C3" s="5" t="inlineStr">
+      <c r="C3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Studi kasus</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">T01, T03</t>
         </is>
       </c>
-      <c r="E3" s="5" t="inlineStr">
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">K01, K02</t>
         </is>
@@ -1039,8 +1062,8 @@
       </c>
       <c r="G3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">[a] B2B menyumbang laba operasi terbesar (98,4), pergudangan paling efisien dengan margin 15%, sedangkan ritel hanya 5% dan ditekan pesaing digital.
-[b] Memperbesar armada ritel berisiko perang tarif. Pergudangan terpadu bersinergi dengan klien B2B dan marginnya tinggi. Saya merekomendasikan pergudangan; risikonya utilisasi gudang rendah pada tahun awal.</t>
+          <t xml:space="preserve">(a) B2B menyumbang laba operasi terbesar (98,4), pergudangan paling efisien dengan margin 15%, sedangkan ritel hanya 5% dan ditekan pesaing digital.
+(b) Memperbesar armada ritel berisiko perang tarif. Pergudangan terpadu bersinergi dengan klien B2B dan marginnya tinggi. Saya merekomendasikan pergudangan; risikonya utilisasi gudang rendah pada tahun awal.</t>
         </is>
       </c>
       <c r="H3" s="3" t="inlineStr">
@@ -1063,48 +1086,52 @@
       </c>
       <c r="M3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Membaca data dan konsep utama dengan benar.</t>
+          <t xml:space="preserve">Membaca data margin ketiga segmen dengan benar dan memberi rekomendasi tegas.</t>
         </is>
       </c>
       <c r="N3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Hubungan sebab-akibat dan dampak keuangan belum dijelaskan.</t>
+          <t xml:space="preserve">Evaluasi pilihan kurang kuantitatif; risiko belum disertai mitigasi.</t>
         </is>
       </c>
       <c r="O3" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Tunjukkan rantai sebab-akibat dan hitung dampak keputusan pada laba.</t>
-        </is>
-      </c>
-      <c r="P3" s="5" t="inlineStr">
+          <t xml:space="preserve">Hitung dampak investasi Rp300 miliar pada laba operasi dan sertakan mitigasi tiap risiko.</t>
+        </is>
+      </c>
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">sedang</t>
         </is>
       </c>
-      <c r="R3" s="5" t="inlineStr">
+      <c r="R3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
       </c>
-      <c r="S3" s="5" t="inlineStr">
+      <c r="S3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
       </c>
-      <c r="T3" s="5" t="inlineStr">
+      <c r="T3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">contoh-penilai (fiktif, untuk uji)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:J12"/>
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:K12"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
@@ -1117,6 +1144,7 @@
     <col min="8" max="8" width="9" customWidth="1"/>
     <col min="9" max="9" width="12" customWidth="1"/>
     <col min="10" max="10" width="70" customWidth="1"/>
+    <col min="11" max="11" width="45" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1170,17 +1198,22 @@
           <t xml:space="preserve">Alasan penilai</t>
         </is>
       </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Alasan koreksi manual</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="4">
         <v>4</v>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-ESA-001</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C1</t>
         </is>
@@ -1199,7 +1232,7 @@
       <c r="H2" s="2">
         <v>3</v>
       </c>
-      <c r="I2" s="5" t="inlineStr">
+      <c r="I2" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
@@ -1214,12 +1247,12 @@
       <c r="A3" s="4">
         <v>4</v>
       </c>
-      <c r="B3" s="5" t="inlineStr">
+      <c r="B3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-ESA-001</t>
         </is>
       </c>
-      <c r="D3" s="5" t="inlineStr">
+      <c r="D3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C2</t>
         </is>
@@ -1238,7 +1271,7 @@
       <c r="H3" s="2">
         <v>3</v>
       </c>
-      <c r="I3" s="5" t="inlineStr">
+      <c r="I3" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
@@ -1253,12 +1286,12 @@
       <c r="A4" s="4">
         <v>4</v>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-ESA-001</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C3</t>
         </is>
@@ -1277,7 +1310,7 @@
       <c r="H4" s="2">
         <v>2</v>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Ya</t>
         </is>
@@ -1285,6 +1318,11 @@
       <c r="J4" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Bukti untuk contoh ukuran per perspektif ditemukan sebagian di jawaban (contoh fiktif).</t>
+        </is>
+      </c>
+      <c r="K4" s="3" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Contoh koreksi: keempat ukuran relevan untuk agribisnis.</t>
         </is>
       </c>
     </row>
@@ -1292,12 +1330,12 @@
       <c r="A5" s="4">
         <v>4</v>
       </c>
-      <c r="B5" s="5" t="inlineStr">
+      <c r="B5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-ESA-001</t>
         </is>
       </c>
-      <c r="D5" s="5" t="inlineStr">
+      <c r="D5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C4</t>
         </is>
@@ -1316,7 +1354,7 @@
       <c r="H5" s="2">
         <v>2</v>
       </c>
-      <c r="I5" s="5" t="inlineStr">
+      <c r="I5" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
@@ -1331,17 +1369,17 @@
       <c r="A6" s="4">
         <v>5</v>
       </c>
-      <c r="B6" s="5" t="inlineStr">
+      <c r="B6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-KAS-001</t>
         </is>
       </c>
-      <c r="C6" s="5" t="inlineStr">
+      <c r="C6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">(a)</t>
         </is>
       </c>
-      <c r="D6" s="5" t="inlineStr">
+      <c r="D6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C1</t>
         </is>
@@ -1360,7 +1398,7 @@
       <c r="H6" s="2">
         <v>3</v>
       </c>
-      <c r="I6" s="5" t="inlineStr">
+      <c r="I6" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
@@ -1375,17 +1413,17 @@
       <c r="A7" s="4">
         <v>5</v>
       </c>
-      <c r="B7" s="5" t="inlineStr">
+      <c r="B7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-KAS-001</t>
         </is>
       </c>
-      <c r="C7" s="5" t="inlineStr">
+      <c r="C7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">(a)</t>
         </is>
       </c>
-      <c r="D7" s="5" t="inlineStr">
+      <c r="D7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C2</t>
         </is>
@@ -1404,7 +1442,7 @@
       <c r="H7" s="2">
         <v>3</v>
       </c>
-      <c r="I7" s="5" t="inlineStr">
+      <c r="I7" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
@@ -1419,17 +1457,17 @@
       <c r="A8" s="4">
         <v>5</v>
       </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="B8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-KAS-001</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
+      <c r="C8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">(a)</t>
         </is>
       </c>
-      <c r="D8" s="5" t="inlineStr">
+      <c r="D8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C3</t>
         </is>
@@ -1448,7 +1486,7 @@
       <c r="H8" s="2">
         <v>2</v>
       </c>
-      <c r="I8" s="5" t="inlineStr">
+      <c r="I8" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
@@ -1463,17 +1501,17 @@
       <c r="A9" s="4">
         <v>5</v>
       </c>
-      <c r="B9" s="5" t="inlineStr">
+      <c r="B9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-KAS-001</t>
         </is>
       </c>
-      <c r="C9" s="5" t="inlineStr">
+      <c r="C9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">(b)</t>
         </is>
       </c>
-      <c r="D9" s="5" t="inlineStr">
+      <c r="D9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C1</t>
         </is>
@@ -1492,7 +1530,7 @@
       <c r="H9" s="2">
         <v>4</v>
       </c>
-      <c r="I9" s="5" t="inlineStr">
+      <c r="I9" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
@@ -1507,17 +1545,17 @@
       <c r="A10" s="4">
         <v>5</v>
       </c>
-      <c r="B10" s="5" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-KAS-001</t>
         </is>
       </c>
-      <c r="C10" s="5" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">(b)</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr">
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C2</t>
         </is>
@@ -1536,7 +1574,7 @@
       <c r="H10" s="2">
         <v>4</v>
       </c>
-      <c r="I10" s="5" t="inlineStr">
+      <c r="I10" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
@@ -1551,17 +1589,17 @@
       <c r="A11" s="4">
         <v>5</v>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-KAS-001</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">(b)</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C3</t>
         </is>
@@ -1580,7 +1618,7 @@
       <c r="H11" s="2">
         <v>2</v>
       </c>
-      <c r="I11" s="5" t="inlineStr">
+      <c r="I11" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
@@ -1595,17 +1633,17 @@
       <c r="A12" s="4">
         <v>5</v>
       </c>
-      <c r="B12" s="5" t="inlineStr">
+      <c r="B12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">DEMO-KAS-001</t>
         </is>
       </c>
-      <c r="C12" s="5" t="inlineStr">
+      <c r="C12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">(b)</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr">
+      <c r="D12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">C4</t>
         </is>
@@ -1624,7 +1662,7 @@
       <c r="H12" s="2">
         <v>2</v>
       </c>
-      <c r="I12" s="5" t="inlineStr">
+      <c r="I12" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Tidak</t>
         </is>
@@ -1636,12 +1674,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:H6"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1683,7 +1725,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capaian (%)</t>
+          <t xml:space="preserve">Capaian</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -1719,8 +1761,8 @@
       <c r="E2" s="2">
         <v>70</v>
       </c>
-      <c r="F2" s="2">
-        <v>65.714286</v>
+      <c r="F2" s="6">
+        <v>0.65714286</v>
       </c>
       <c r="G2" s="5" t="inlineStr">
         <is>
@@ -1755,8 +1797,8 @@
       <c r="E3" s="2">
         <v>30</v>
       </c>
-      <c r="F3" s="2">
-        <v>78.333333</v>
+      <c r="F3" s="6">
+        <v>0.7833333299999999</v>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
@@ -1791,8 +1833,8 @@
       <c r="E4" s="2">
         <v>30</v>
       </c>
-      <c r="F4" s="2">
-        <v>78.333333</v>
+      <c r="F4" s="6">
+        <v>0.7833333299999999</v>
       </c>
       <c r="G4" s="5" t="inlineStr">
         <is>
@@ -1827,8 +1869,8 @@
       <c r="E5" s="2">
         <v>40</v>
       </c>
-      <c r="F5" s="2">
-        <v>56.25</v>
+      <c r="F5" s="6">
+        <v>0.5625</v>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
@@ -1863,8 +1905,8 @@
       <c r="E6" s="2">
         <v>30</v>
       </c>
-      <c r="F6" s="2">
-        <v>78.333333</v>
+      <c r="F6" s="6">
+        <v>0.7833333299999999</v>
       </c>
       <c r="G6" s="5" t="inlineStr">
         <is>
@@ -1878,12 +1920,16 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:E9"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -1912,7 +1958,7 @@
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t xml:space="preserve">Capaian (%)</t>
+          <t xml:space="preserve">Capaian</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
@@ -1937,12 +1983,12 @@
           <t xml:space="preserve">Pengukuran kinerja strategis</t>
         </is>
       </c>
-      <c r="D2" s="2">
-        <v>56.25</v>
+      <c r="D2" s="6">
+        <v>0.5625</v>
       </c>
       <c r="E2" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pelajari ulang konsep: Balanced scorecard dan strategy map; Balanced scorecard.</t>
+          <t xml:space="preserve">Pelajari ulang konsep: Balanced scorecard dan strategy map.</t>
         </is>
       </c>
     </row>
@@ -1962,8 +2008,8 @@
           <t xml:space="preserve">Pengukuran kinerja strategis</t>
         </is>
       </c>
-      <c r="D3" s="2">
-        <v>56.25</v>
+      <c r="D3" s="6">
+        <v>0.5625</v>
       </c>
       <c r="E3" s="3" t="inlineStr">
         <is>
@@ -1987,12 +2033,12 @@
           <t xml:space="preserve">Pengukuran kinerja strategis</t>
         </is>
       </c>
-      <c r="D4" s="2">
-        <v>56.25</v>
+      <c r="D4" s="6">
+        <v>0.5625</v>
       </c>
       <c r="E4" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Saran penilai untuk Soal 4: Tunjukkan rantai sebab-akibat dan hitung dampak keputusan pada laba.</t>
+          <t xml:space="preserve">Saran penilai untuk Soal 4: Gambarkan strategy map: pembelajaran -&gt; proses internal -&gt; pelanggan -&gt; keuangan.</t>
         </is>
       </c>
     </row>
@@ -2012,8 +2058,8 @@
           <t xml:space="preserve">Pengukuran kinerja strategis</t>
         </is>
       </c>
-      <c r="D5" s="2">
-        <v>56.25</v>
+      <c r="D5" s="6">
+        <v>0.5625</v>
       </c>
       <c r="E5" s="3" t="inlineStr">
         <is>
@@ -2037,12 +2083,12 @@
           <t xml:space="preserve">Menganalisis dan mengevaluasi strategi</t>
         </is>
       </c>
-      <c r="D6" s="2">
-        <v>65.714286</v>
+      <c r="D6" s="6">
+        <v>0.65714286</v>
       </c>
       <c r="E6" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Pelajari ulang konsep: Balanced scorecard dan strategy map; Balanced scorecard; Analisis portofolio bisnis; Keunggulan bersaing Porter.</t>
+          <t xml:space="preserve">Pelajari ulang konsep: Balanced scorecard dan strategy map; Analisis portofolio bisnis; Keunggulan bersaing Porter.</t>
         </is>
       </c>
     </row>
@@ -2062,8 +2108,8 @@
           <t xml:space="preserve">Menganalisis dan mengevaluasi strategi</t>
         </is>
       </c>
-      <c r="D7" s="2">
-        <v>65.714286</v>
+      <c r="D7" s="6">
+        <v>0.65714286</v>
       </c>
       <c r="E7" s="3" t="inlineStr">
         <is>
@@ -2087,12 +2133,12 @@
           <t xml:space="preserve">Menganalisis dan mengevaluasi strategi</t>
         </is>
       </c>
-      <c r="D8" s="2">
-        <v>65.714286</v>
+      <c r="D8" s="6">
+        <v>0.65714286</v>
       </c>
       <c r="E8" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Saran penilai untuk Soal 4: Tunjukkan rantai sebab-akibat dan hitung dampak keputusan pada laba.</t>
+          <t xml:space="preserve">Saran penilai untuk Soal 4: Gambarkan strategy map: pembelajaran -&gt; proses internal -&gt; pelanggan -&gt; keuangan.</t>
         </is>
       </c>
     </row>
@@ -2112,22 +2158,26 @@
           <t xml:space="preserve">Menganalisis dan mengevaluasi strategi</t>
         </is>
       </c>
-      <c r="D9" s="2">
-        <v>65.714286</v>
+      <c r="D9" s="6">
+        <v>0.65714286</v>
       </c>
       <c r="E9" s="3" t="inlineStr">
         <is>
-          <t xml:space="preserve">Saran penilai untuk Soal 5: Tunjukkan rantai sebab-akibat dan hitung dampak keputusan pada laba.</t>
+          <t xml:space="preserve">Saran penilai untuk Soal 5: Hitung dampak investasi Rp300 miliar pada laba operasi dan sertakan mitigasi tiap risiko.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
   <dimension ref="A1:F3"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
@@ -2172,10 +2222,8 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">16 Oktober 2026 pukul 08.25</t>
-        </is>
+      <c r="A2" s="7">
+        <v>46311.350694444445</v>
       </c>
       <c r="B2" s="5" t="inlineStr">
         <is>
@@ -2184,7 +2232,7 @@
       </c>
       <c r="C2" s="5" t="inlineStr">
         <is>
-          <t xml:space="preserve">demo-20261017-3919b7e3</t>
+          <t xml:space="preserve">demo-20261016-3919b7e3</t>
         </is>
       </c>
       <c r="D2" s="2">
@@ -2200,10 +2248,8 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="5" t="inlineStr">
-        <is>
-          <t xml:space="preserve">17 Oktober 2026 pukul 08.25</t>
-        </is>
+      <c r="A3" s="7">
+        <v>46312.350694444445</v>
       </c>
       <c r="B3" s="5" t="inlineStr">
         <is>
@@ -2228,6 +2274,7 @@
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageMargins left="0.5" right="0.5" top="0.6" bottom="0.6" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="landscape" fitToWidth="1" fitToHeight="0"/>
 </worksheet>
 </file>
</xml_diff>